<commit_message>
add column to applications.xlsx to track the number of times a job has been applied to
</commit_message>
<xml_diff>
--- a/client/src/resumix_client/resources/applications.xlsx
+++ b/client/src/resumix_client/resources/applications.xlsx
@@ -10,7 +10,7 @@
     <sheet name="applications" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'applications'!$A$1:$F$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'applications'!$A$1:$G$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -435,6 +435,7 @@
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="50" customWidth="1" min="5" max="5"/>
     <col width="46" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -468,12 +469,17 @@
           <t>webLink</t>
         </is>
       </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>cv_path</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F1"/>
+  <autoFilter ref="A1:G1"/>
   <dataValidations count="1">
     <dataValidation sqref="D2:D500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Unknown status" error="Pick one of: not applied, applied, wait 1st interview, wait follow up" type="list">
-      <formula1>"not applied,applied,wait 1st interview,wait follow up"</formula1>
+      <formula1>"not applied,applied,wait 1st interview,wait follow up,discarded"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>